<commit_message>
feat: add purchase, audit and contract checks
Add five SAM toolkit templates (proof of purchase, acquisition gate,
invoice verification, savings report, contract terms) and an audit
response method with demo data and practicum exercise 08.

Wire the new checks into the existing checklists, SOPs, skills, router,
agent and lifecycle rules so governance work uses them.

Fixes #29

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011jjas23m3NwpgZMZpEjChK
</commit_message>
<xml_diff>
--- a/site/docs/app-governance/method.xlsx
+++ b/site/docs/app-governance/method.xlsx
@@ -61,7 +61,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="60" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="2" max="2" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -163,10 +163,70 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">Answer a publisher's audit letter, or test the audit response plan before one arrives: check proofs of purchase against installs and brief counsel</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">audit-response</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Buy new software or approve a purchase</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">rationalization, with sam-toolkit/acquisition-gate-checklist.md (the gate runs first and sends an AI tool to ai-intake)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Check invoices before payment, or report what the practice saved</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">rationalization, with sam-toolkit/invoice-verification.csv and sam-toolkit/savings-report.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Read contract terms or prepare for an upcoming renewal</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">rationalization, with sam-toolkit/contract-terms-check.csv and sam-toolkit/renewal-calendar.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Check license entitlement against purchase records as a routine check</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">itam-maturity, with sam-toolkit/proof-of-purchase-check.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="0">
+        <is>
           <t xml:space="preserve">Practice for CAMP, CSAM, CHAMP, AIGP, ITIL 4 Foundation, or the IAM Certificate</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="0">
+      <c r="B14" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">cert-prep</t>
         </is>

</xml_diff>

<commit_message>
feat: add software-lifecycle method
Adds software lifecycle as the ninth tool: a method, checklist, SOP, platform guide, Copilot test, template and synthetic example. It runs the offline software-lifecycle tool pinned to v0.7.0 and relays summary counts only. The Claude app and ChatGPT are marked unsupported.

Fixes #33

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011jjas1nbTyQijgNwgRkSB9
</commit_message>
<xml_diff>
--- a/site/docs/app-governance/method.xlsx
+++ b/site/docs/app-governance/method.xlsx
@@ -163,70 +163,82 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Answer a publisher's audit letter, or test the audit response plan before one arrives: check proofs of purchase against installs and brief counsel</t>
+          <t xml:space="preserve">Find installed software past or near end of life, with a CISA KEV needs-review flag, from a software inventory export: counts only, run on the person's own machine</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">audit-response</t>
+          <t xml:space="preserve">software-lifecycle</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Buy new software or approve a purchase</t>
+          <t xml:space="preserve">Answer a publisher's audit letter, or test the audit response plan before one arrives: check proofs of purchase against installs and brief counsel</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">rationalization, with sam-toolkit/acquisition-gate-checklist.md (the gate runs first and sends an AI tool to ai-intake)</t>
+          <t xml:space="preserve">audit-response</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Check invoices before payment, or report what the practice saved</t>
+          <t xml:space="preserve">Buy new software or approve a purchase</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">rationalization, with sam-toolkit/invoice-verification.csv and sam-toolkit/savings-report.csv</t>
+          <t xml:space="preserve">rationalization, with sam-toolkit/acquisition-gate-checklist.md (the gate runs first and sends an AI tool to ai-intake)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Read contract terms or prepare for an upcoming renewal</t>
+          <t xml:space="preserve">Check invoices before payment, or report what the practice saved</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">rationalization, with sam-toolkit/contract-terms-check.csv and sam-toolkit/renewal-calendar.csv</t>
+          <t xml:space="preserve">rationalization, with sam-toolkit/invoice-verification.csv and sam-toolkit/savings-report.csv</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Check license entitlement against purchase records as a routine check</t>
+          <t xml:space="preserve">Read contract terms or prepare for an upcoming renewal</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">itam-maturity, with sam-toolkit/proof-of-purchase-check.csv</t>
+          <t xml:space="preserve">rationalization, with sam-toolkit/contract-terms-check.csv and sam-toolkit/renewal-calendar.csv</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">Check license entitlement against purchase records as a routine check</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">itam-maturity, with sam-toolkit/proof-of-purchase-check.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="0">
+        <is>
           <t xml:space="preserve">Practice for CAMP, CSAM, CHAMP, AIGP, ITIL 4 Foundation, or the IAM Certificate</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="0">
+      <c r="B15" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">cert-prep</t>
         </is>

</xml_diff>